<commit_message>
docs: update based on s3,ddb and no efs, remove turbo example since we next build locally now
</commit_message>
<xml_diff>
--- a/docs/usage.xlsx
+++ b/docs/usage.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stickb/Code/cdk-nextjs/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F01743A-8774-F24E-BEE0-52FBE8E8BB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5CEB85-10E0-CE45-8D60-86A16835F264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3220" yWindow="2140" windowWidth="28040" windowHeight="17440" xr2:uid="{3F8BC154-5623-A945-9212-C702D7AAC795}"/>
+    <workbookView xWindow="3220" yWindow="2140" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{3F8BC154-5623-A945-9212-C702D7AAC795}"/>
   </bookViews>
   <sheets>
     <sheet name="NextjsGlobalFunctions" sheetId="1" r:id="rId1"/>
     <sheet name="NextjsGlobalContainers" sheetId="3" r:id="rId2"/>
     <sheet name="NextjsRegionalContainers" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,6 +29,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="49">
   <si>
     <t>Assumptions</t>
   </si>
@@ -108,24 +109,6 @@
     <t>CloudFront Requests</t>
   </si>
   <si>
-    <t>S3 Storage</t>
-  </si>
-  <si>
-    <t>S3 GET Requests</t>
-  </si>
-  <si>
-    <t>S3 Data Transfer Out</t>
-  </si>
-  <si>
-    <t>EFS Storage</t>
-  </si>
-  <si>
-    <t>EFS Read Throughput</t>
-  </si>
-  <si>
-    <t>EFS Write Throughput</t>
-  </si>
-  <si>
     <t>Dynamic Cache Write %</t>
   </si>
   <si>
@@ -175,6 +158,33 @@
   </si>
   <si>
     <t>Pages Visited Per Month Per User</t>
+  </si>
+  <si>
+    <t>Static Assets - S3 GET Requests</t>
+  </si>
+  <si>
+    <t>Static Assets - S3 Storage</t>
+  </si>
+  <si>
+    <t>Cache - S3 PUT Requests</t>
+  </si>
+  <si>
+    <t>Cache - S3 GET Requests</t>
+  </si>
+  <si>
+    <t>Cache - DDB RCU</t>
+  </si>
+  <si>
+    <t>Cache - DDB Storage</t>
+  </si>
+  <si>
+    <t>Cache - DDB WCU</t>
+  </si>
+  <si>
+    <t>Dynamic Revalidate Tag %</t>
+  </si>
+  <si>
+    <t>Cache - S3 Storage</t>
   </si>
 </sst>
 </file>
@@ -231,12 +241,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -256,9 +266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -296,7 +306,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -402,7 +412,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -544,7 +554,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -561,34 +571,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -596,20 +606,20 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>1000</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <f>$B$3*$B$4*$B$10</f>
         <v>500000</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>100</v>
@@ -617,8 +627,8 @@
       <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="4">
-        <f>$F$3*$B$15/1000*$B$16</f>
+      <c r="F4" s="3">
+        <f>$F$3*$B$14/1000*$B$15</f>
         <v>150000</v>
       </c>
       <c r="G4" t="s">
@@ -638,7 +648,7 @@
       <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <f>$B$3*$B$4*($B$10+$B$7)/1000000</f>
         <v>2</v>
       </c>
@@ -648,15 +658,15 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <v>0.05</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="4">
+        <v>25</v>
+      </c>
+      <c r="F6" s="3">
         <f>$B$3*$B$4*($B$7+$B$10)*$B$5/1000000</f>
         <v>100</v>
       </c>
@@ -672,9 +682,9 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="4">
+        <v>26</v>
+      </c>
+      <c r="F7" s="3">
         <f>$F$5*1000000*$B$6*$B$5/1000000</f>
         <v>5</v>
       </c>
@@ -690,7 +700,7 @@
         <v>0.5</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="F8">
         <f>$B$9</f>
@@ -711,9 +721,9 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="4">
+        <v>40</v>
+      </c>
+      <c r="F9" s="3">
         <f>$B$3*$B$4*$B$7*(1-$B$8)</f>
         <v>750000</v>
       </c>
@@ -726,11 +736,10 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="4">
-        <f>$F$9*$B$5/1000000</f>
-        <v>37.5</v>
+        <v>48</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
       </c>
       <c r="G10" t="s">
         <v>8</v>
@@ -738,92 +747,96 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>0.5</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11">
-        <f>$B$13</f>
-        <v>10</v>
-      </c>
-      <c r="G11" t="s">
-        <v>8</v>
+        <v>42</v>
+      </c>
+      <c r="F11" s="3">
+        <f>$F$3*$B$12</f>
+        <v>25000</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B12">
         <v>0.05</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="4">
-        <f>$F$3*$B$11*$B$14/1000000</f>
-        <v>25</v>
-      </c>
-      <c r="G12" t="s">
-        <v>8</v>
+        <v>43</v>
+      </c>
+      <c r="F12" s="3">
+        <f>$F$3*$B$11</f>
+        <v>250000</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="4">
-        <f>$F$3*$B$12*$B$14/1000000</f>
-        <v>2.5</v>
-      </c>
-      <c r="G13" t="s">
-        <v>8</v>
+        <v>44</v>
+      </c>
+      <c r="F13" s="3">
+        <f>$F$3*$B$16</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C14" t="s">
-        <v>4</v>
+        <v>20</v>
+      </c>
+      <c r="E14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="3">
+        <f>$F$3*$B$16</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B15">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>8</v>
+      </c>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="B16">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEEA12D8-FAB4-8F44-BA90-F8D535F6EDBB}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
@@ -847,34 +860,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -882,33 +895,33 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>1000</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="3">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2">
         <f>ROUNDUP($B$3*$B$4*$B$10/(24*60*60)/$B$17, 0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="4">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3">
         <f>$B$3*$B$4*$B$10/24*$B$5/1000000</f>
         <v>1.0416666666666665</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -922,19 +935,19 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="4">
+        <v>34</v>
+      </c>
+      <c r="F5" s="3">
         <f>B3*B4*B10/(24*60*60)</f>
         <v>5.7870370370370372</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <v>0.05</v>
@@ -942,7 +955,7 @@
       <c r="E6" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <f>$B$3*$B$4*($B$10+$B$7)/1000000</f>
         <v>2</v>
       </c>
@@ -958,9 +971,9 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="4">
+        <v>25</v>
+      </c>
+      <c r="F7" s="3">
         <f>$B$3*$B$4*($B$7+$B$10)*$B$5/1000000</f>
         <v>100</v>
       </c>
@@ -976,9 +989,9 @@
         <v>0.5</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" s="4">
+        <v>26</v>
+      </c>
+      <c r="F8" s="3">
         <f>$F$6*1000000*$B$6*$B$5/1000000</f>
         <v>5</v>
       </c>
@@ -997,7 +1010,7 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="F9">
         <f>$B$9</f>
@@ -1015,47 +1028,41 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="4">
+        <v>40</v>
+      </c>
+      <c r="F10" s="3">
         <f>$B$3*$B$4*$B$7*(1-$B$8)</f>
         <v>750000</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>0.5</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="4">
-        <f>$F$10*$B$5/1000000</f>
-        <v>37.5</v>
-      </c>
-      <c r="G11" t="s">
-        <v>8</v>
+        <v>42</v>
+      </c>
+      <c r="F11" s="3">
+        <f>$B$3*$B$4*$B$10*$B$12</f>
+        <v>25000</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B12">
         <v>0.05</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12">
-        <f>$B$13</f>
-        <v>10</v>
-      </c>
-      <c r="G12" t="s">
-        <v>8</v>
+        <v>43</v>
+      </c>
+      <c r="F12" s="3">
+        <f>$B$3*$B$4*$B$10*$B$11</f>
+        <v>250000</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1069,14 +1076,11 @@
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="4">
-        <f>$B$3*$B$4*$B$10*$B$11*$B$14/1000000</f>
-        <v>25</v>
-      </c>
-      <c r="G13" t="s">
-        <v>8</v>
+        <v>44</v>
+      </c>
+      <c r="F13" s="3">
+        <f>$B$3*$B$4*$B$10*$B$19</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1090,30 +1094,36 @@
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="4">
-        <f>$B$3*$B$4*$B$10*$B$12*B14/1000000</f>
-        <v>2.5</v>
-      </c>
-      <c r="G14" t="s">
-        <v>8</v>
+        <v>46</v>
+      </c>
+      <c r="F14" s="3">
+        <f>$B$3*$B$4*$B$10*$B$19</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -1124,7 +1134,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B17">
         <v>100</v>
@@ -1132,13 +1142,21 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -1153,7 +1171,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B543F87-360B-F345-8BC3-38BB33A55C0F}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
@@ -1162,34 +1180,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1197,33 +1215,33 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>1000</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="3">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2">
         <f>ROUNDUP($B$3*$B$4*($B$6+$B$8)/(24*60*60)/$B$15, 0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="4">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3">
         <f>$B$3*$B$4*($B$6+$B$8)/24*$B$5/1000000</f>
         <v>4.1666666666666661</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1237,14 +1255,14 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="4">
+        <v>34</v>
+      </c>
+      <c r="F5" s="3">
         <f>$B$3*$B$4*($B$6+$B$8)/(24*60*60)</f>
         <v>23.148148148148149</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1255,14 +1273,11 @@
         <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6">
-        <f>$B$11</f>
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>8</v>
+        <v>42</v>
+      </c>
+      <c r="F6" s="3">
+        <f>$B$3*$B$4*$B$8*$B$10</f>
+        <v>25000</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -1276,14 +1291,11 @@
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="4">
-        <f>$B$3*$B$4*$B$8*$B$9*$B$12/1000000</f>
-        <v>25</v>
-      </c>
-      <c r="G7" t="s">
-        <v>8</v>
+        <v>43</v>
+      </c>
+      <c r="F7" s="3">
+        <f>$B$3*$B$4*$B$8*$B$9</f>
+        <v>250000</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -1294,32 +1306,44 @@
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="4">
-        <f>$B$3*$B$4*$B$8*$B$10*$B$12/1000000</f>
-        <v>2.5</v>
-      </c>
-      <c r="G8" t="s">
-        <v>8</v>
+        <v>44</v>
+      </c>
+      <c r="F8" s="3">
+        <f>$B$3*$B$4*$B$8*$B$17</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B9">
         <v>0.5</v>
       </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="3">
+        <f>$B$3*$B$4*$B$8*$B$17</f>
+        <v>5000</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B10">
         <v>0.05</v>
       </c>
-      <c r="F10" s="4"/>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="G10" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1331,7 +1355,6 @@
       <c r="C11" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -1346,19 +1369,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="4"/>
+        <v>30</v>
+      </c>
+      <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -1366,11 +1389,11 @@
       <c r="C14" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="4"/>
+      <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B15">
         <v>100</v>
@@ -1378,13 +1401,21 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>